<commit_message>
upgrade raha and 1.1.0 features
</commit_message>
<xml_diff>
--- a/voyah-voice-test/research/Raha-Action-Catalog.xlsx
+++ b/voyah-voice-test/research/Raha-Action-Catalog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nahid\Documents\voyah-iran\voyah-voice-test\research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18C74950-CBDA-4B4C-971A-A2375C2FE6E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1686D5F-944C-412A-A61E-40420C033C60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9088" uniqueCount="2837">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9088" uniqueCount="2849">
   <si>
     <t>اکشن</t>
   </si>
@@ -8538,6 +8538,42 @@
   </si>
   <si>
     <t>تشخیص جمله اضافه شد؛ اجرای کنترل مستقیم آینه در H97 تأیید نشده و هیچ فرمانی ارسال نمی‌شود. گزینهٔ جمع‌شدن خودکار جایگزین آن نشده است.</t>
+  </si>
+  <si>
+    <t>فاز ۷: تشخیص جمله و اجرای کنترل اصلی منوی خودرو اضافه شد؛ فقط کنترل قابل‌نمایش و فعال. نیازمند تست خودرو.</t>
+  </si>
+  <si>
+    <t>فاز ۷: روشن/خاموش و حساسیت کم/متوسط/زیاد از کنترل اصلی منو؛ تأیید خاموش‌کردن حفظ شده. نیازمند تست خودرو.</t>
+  </si>
+  <si>
+    <t>فاز ۷: کنترل اصلی ترمز اضطراری؛ تأیید خاموش‌کردن باید در پنجره خود خودرو انجام شود. نیازمند تست خودرو.</t>
+  </si>
+  <si>
+    <t>فاز ۷ ناقص: خاموش، هشدار و حفظ خط پیاده شد؛ مسیر مستقل مرکز خط تأیید نشده و اجرا نمی‌شود. زرد باقی ماند. نیازمند تست خودرو.</t>
+  </si>
+  <si>
+    <t>فاز ۷: روشن/خاموش و حساسیت عادی یا حساس (حداقل/حداکثر)؛ شروط اصلی DMS حفظ می‌شوند. نیازمند تست خودرو.</t>
+  </si>
+  <si>
+    <t>فاز ۷: روشنایی مرکزی/شاگرد/پشت‌آمپر/همه؛ درصد مطلق یا تغییر ۱۰ درصدی. همگام‌سازی اصلی خودرو حفظ می‌شود. نیازمند تست خودرو.</t>
+  </si>
+  <si>
+    <t>فاز ۷: حالت روشنایی روز/شب/خودکار از منوی اصلی نمایشگر. نیازمند تست خودرو.</t>
+  </si>
+  <si>
+    <t>فاز ۷: قفل نمایشگر عقب از کنترل واقعی منو؛ فقط اگر آن کنترل روی خودرو موجود باشد. نیازمند تست خودرو.</t>
+  </si>
+  <si>
+    <t>فاز ۷: کانال‌های موسیقی، تماس، مسیریاب، دستیار صوتی و سیستم با AudioPolicy خودرو؛ بازه واقعی دستگاه بررسی می‌شود. نیازمند تست خودرو.</t>
+  </si>
+  <si>
+    <t>فاز ۷: ارسال کلید رسانه به پلیر فعال سیستم؛ رها پیش از فرمان فوکوس صدا را آزاد می‌کند. نیازمند تست خودرو.</t>
+  </si>
+  <si>
+    <t>فاز ۷: دوربین پیش‌فرض از مسیر اصلی اپ Camera؛ انتخاب نمای خاص اضافه نشده؛ شروط اشغال دوربین و دنده‌عقب حفظ می‌شوند. نیازمند تست خودرو.</t>
+  </si>
+  <si>
+    <t>فاز ۷: توقف ضبط با رویداد اصلی اپ Camera؛ بدون بازکردن دوباره برنامه و بدون تبدیل توقف به شروع. نیازمند تست خودرو.</t>
   </si>
 </sst>
 </file>
@@ -8704,7 +8740,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -8780,84 +8816,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -12291,7 +12249,7 @@
       </c>
     </row>
     <row r="120" spans="1:8" ht="56" customHeight="1">
-      <c r="A120" s="28" t="s">
+      <c r="A120" s="6" t="s">
         <v>536</v>
       </c>
       <c r="B120" s="5" t="s">
@@ -12312,14 +12270,12 @@
       <c r="G120" s="5" t="s">
         <v>540</v>
       </c>
-      <c r="H120" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷: تشخیص جمله و اجرای کنترل اصلی منوی خودرو اضافه شد؛ فقط کنترل قابل‌نمایش و فعال. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H120" s="5" t="s">
+        <v>2837</v>
       </c>
     </row>
     <row r="121" spans="1:8" ht="56" customHeight="1">
-      <c r="A121" s="29" t="s">
+      <c r="A121" s="6" t="s">
         <v>542</v>
       </c>
       <c r="B121" s="1" t="s">
@@ -12340,14 +12296,12 @@
       <c r="G121" s="1" t="s">
         <v>546</v>
       </c>
-      <c r="H121" s="1" t="inlineStr">
-        <is>
-          <t>فاز ۷: روشن/خاموش و حساسیت کم/متوسط/زیاد از کنترل اصلی منو؛ تأیید خاموش‌کردن حفظ شده. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H121" s="1" t="s">
+        <v>2838</v>
       </c>
     </row>
     <row r="122" spans="1:8" ht="56" customHeight="1">
-      <c r="A122" s="30" t="s">
+      <c r="A122" s="6" t="s">
         <v>547</v>
       </c>
       <c r="B122" s="5" t="s">
@@ -12368,14 +12322,12 @@
       <c r="G122" s="5" t="s">
         <v>550</v>
       </c>
-      <c r="H122" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷: تشخیص جمله و اجرای کنترل اصلی منوی خودرو اضافه شد؛ فقط کنترل قابل‌نمایش و فعال. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H122" s="5" t="s">
+        <v>2837</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="56" customHeight="1">
-      <c r="A123" s="31" t="s">
+      <c r="A123" s="6" t="s">
         <v>551</v>
       </c>
       <c r="B123" s="1" t="s">
@@ -12396,14 +12348,12 @@
       <c r="G123" s="1" t="s">
         <v>554</v>
       </c>
-      <c r="H123" s="1" t="inlineStr">
-        <is>
-          <t>فاز ۷: تشخیص جمله و اجرای کنترل اصلی منوی خودرو اضافه شد؛ فقط کنترل قابل‌نمایش و فعال. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H123" s="1" t="s">
+        <v>2837</v>
       </c>
     </row>
     <row r="124" spans="1:8" ht="56" customHeight="1">
-      <c r="A124" s="32" t="s">
+      <c r="A124" s="6" t="s">
         <v>555</v>
       </c>
       <c r="B124" s="5" t="s">
@@ -12424,14 +12374,12 @@
       <c r="G124" s="5" t="s">
         <v>558</v>
       </c>
-      <c r="H124" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷: کنترل اصلی ترمز اضطراری؛ تأیید خاموش‌کردن باید در پنجره خود خودرو انجام شود. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H124" s="5" t="s">
+        <v>2839</v>
       </c>
     </row>
     <row r="125" spans="1:8" ht="56" customHeight="1">
-      <c r="A125" s="33" t="s">
+      <c r="A125" s="6" t="s">
         <v>559</v>
       </c>
       <c r="B125" s="1" t="s">
@@ -12452,14 +12400,12 @@
       <c r="G125" s="1" t="s">
         <v>562</v>
       </c>
-      <c r="H125" s="1" t="inlineStr">
-        <is>
-          <t>فاز ۷: تشخیص جمله و اجرای کنترل اصلی منوی خودرو اضافه شد؛ فقط کنترل قابل‌نمایش و فعال. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H125" s="1" t="s">
+        <v>2837</v>
       </c>
     </row>
     <row r="126" spans="1:8" ht="56" customHeight="1">
-      <c r="A126" s="21" t="s">
+      <c r="A126" s="22" t="s">
         <v>563</v>
       </c>
       <c r="B126" s="5" t="s">
@@ -12480,10 +12426,8 @@
       <c r="G126" s="5" t="s">
         <v>567</v>
       </c>
-      <c r="H126" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷ ناقص: خاموش، هشدار و حفظ خط پیاده شد؛ مسیر مستقل مرکز خط تأیید نشده و اجرا نمی‌شود. زرد باقی ماند. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H126" s="5" t="s">
+        <v>2840</v>
       </c>
     </row>
     <row r="127" spans="1:8" ht="56" customHeight="1">
@@ -12513,7 +12457,7 @@
       </c>
     </row>
     <row r="128" spans="1:8" ht="56" customHeight="1">
-      <c r="A128" s="34" t="s">
+      <c r="A128" s="6" t="s">
         <v>572</v>
       </c>
       <c r="B128" s="5" t="s">
@@ -12534,10 +12478,8 @@
       <c r="G128" s="5" t="s">
         <v>575</v>
       </c>
-      <c r="H128" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷: روشن/خاموش و حساسیت عادی یا حساس (حداقل/حداکثر)؛ شروط اصلی DMS حفظ می‌شوند. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H128" s="5" t="s">
+        <v>2841</v>
       </c>
     </row>
     <row r="129" spans="1:8" ht="56" customHeight="1">
@@ -12567,7 +12509,7 @@
       </c>
     </row>
     <row r="130" spans="1:8" ht="56" customHeight="1">
-      <c r="A130" s="35" t="s">
+      <c r="A130" s="6" t="s">
         <v>580</v>
       </c>
       <c r="B130" s="5" t="s">
@@ -12588,10 +12530,8 @@
       <c r="G130" s="5" t="s">
         <v>583</v>
       </c>
-      <c r="H130" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷: تشخیص جمله و اجرای کنترل اصلی منوی خودرو اضافه شد؛ فقط کنترل قابل‌نمایش و فعال. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H130" s="5" t="s">
+        <v>2837</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="56" customHeight="1">
@@ -12855,7 +12795,7 @@
       </c>
     </row>
     <row r="141" spans="1:8" ht="56" customHeight="1">
-      <c r="A141" s="36" t="s">
+      <c r="A141" s="6" t="s">
         <v>625</v>
       </c>
       <c r="B141" s="1" t="s">
@@ -12876,14 +12816,12 @@
       <c r="G141" s="1" t="s">
         <v>628</v>
       </c>
-      <c r="H141" s="1" t="inlineStr">
-        <is>
-          <t>فاز ۷: تشخیص جمله و اجرای کنترل اصلی منوی خودرو اضافه شد؛ فقط کنترل قابل‌نمایش و فعال. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H141" s="1" t="s">
+        <v>2837</v>
       </c>
     </row>
     <row r="142" spans="1:8" ht="56" customHeight="1">
-      <c r="A142" s="37" t="s">
+      <c r="A142" s="6" t="s">
         <v>629</v>
       </c>
       <c r="B142" s="5" t="s">
@@ -12904,14 +12842,12 @@
       <c r="G142" s="5" t="s">
         <v>632</v>
       </c>
-      <c r="H142" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷: تشخیص جمله و اجرای کنترل اصلی منوی خودرو اضافه شد؛ فقط کنترل قابل‌نمایش و فعال. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H142" s="5" t="s">
+        <v>2837</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="56" customHeight="1">
-      <c r="A143" s="38" t="s">
+      <c r="A143" s="6" t="s">
         <v>633</v>
       </c>
       <c r="B143" s="1" t="s">
@@ -12932,10 +12868,8 @@
       <c r="G143" s="1" t="s">
         <v>636</v>
       </c>
-      <c r="H143" s="1" t="inlineStr">
-        <is>
-          <t>فاز ۷: تشخیص جمله و اجرای کنترل اصلی منوی خودرو اضافه شد؛ فقط کنترل قابل‌نمایش و فعال. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H143" s="1" t="s">
+        <v>2837</v>
       </c>
     </row>
     <row r="144" spans="1:8" ht="56" customHeight="1">
@@ -13173,7 +13107,7 @@
       </c>
     </row>
     <row r="153" spans="1:8" ht="56" customHeight="1">
-      <c r="A153" s="39" t="s">
+      <c r="A153" s="6" t="s">
         <v>677</v>
       </c>
       <c r="B153" s="1" t="s">
@@ -13194,10 +13128,8 @@
       <c r="G153" s="1" t="s">
         <v>681</v>
       </c>
-      <c r="H153" s="1" t="inlineStr">
-        <is>
-          <t>فاز ۷: تشخیص جمله و اجرای کنترل اصلی منوی خودرو اضافه شد؛ فقط کنترل قابل‌نمایش و فعال. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H153" s="1" t="s">
+        <v>2837</v>
       </c>
     </row>
     <row r="154" spans="1:8" ht="56" customHeight="1">
@@ -13253,7 +13185,7 @@
       </c>
     </row>
     <row r="156" spans="1:8" ht="56" customHeight="1">
-      <c r="A156" s="40" t="s">
+      <c r="A156" s="6" t="s">
         <v>691</v>
       </c>
       <c r="B156" s="5" t="s">
@@ -13274,14 +13206,12 @@
       <c r="G156" s="5" t="s">
         <v>696</v>
       </c>
-      <c r="H156" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷: روشنایی مرکزی/شاگرد/پشت‌آمپر/همه؛ درصد مطلق یا تغییر ۱۰ درصدی. همگام‌سازی اصلی خودرو حفظ می‌شود. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H156" s="5" t="s">
+        <v>2842</v>
       </c>
     </row>
     <row r="157" spans="1:8" ht="56" customHeight="1">
-      <c r="A157" s="41" t="s">
+      <c r="A157" s="6" t="s">
         <v>697</v>
       </c>
       <c r="B157" s="1" t="s">
@@ -13302,10 +13232,8 @@
       <c r="G157" s="1" t="s">
         <v>701</v>
       </c>
-      <c r="H157" s="1" t="inlineStr">
-        <is>
-          <t>فاز ۷: حالت روشنایی روز/شب/خودکار از منوی اصلی نمایشگر. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H157" s="1" t="s">
+        <v>2843</v>
       </c>
     </row>
     <row r="158" spans="1:8" ht="56" customHeight="1">
@@ -13777,7 +13705,7 @@
       </c>
     </row>
     <row r="176" spans="1:8" ht="56" customHeight="1">
-      <c r="A176" s="42" t="s">
+      <c r="A176" s="6" t="s">
         <v>786</v>
       </c>
       <c r="B176" s="5" t="s">
@@ -13798,14 +13726,12 @@
       <c r="G176" s="5" t="s">
         <v>789</v>
       </c>
-      <c r="H176" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷: قفل نمایشگر عقب از کنترل واقعی منو؛ فقط اگر آن کنترل روی خودرو موجود باشد. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H176" s="5" t="s">
+        <v>2844</v>
       </c>
     </row>
     <row r="177" spans="1:8" ht="56" customHeight="1">
-      <c r="A177" s="43" t="s">
+      <c r="A177" s="6" t="s">
         <v>790</v>
       </c>
       <c r="B177" s="1" t="s">
@@ -13826,14 +13752,12 @@
       <c r="G177" s="1" t="s">
         <v>795</v>
       </c>
-      <c r="H177" s="1" t="inlineStr">
-        <is>
-          <t>فاز ۷: کانال‌های موسیقی، تماس، مسیریاب، دستیار صوتی و سیستم با AudioPolicy خودرو؛ بازه واقعی دستگاه بررسی می‌شود. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H177" s="1" t="s">
+        <v>2845</v>
       </c>
     </row>
     <row r="178" spans="1:8" ht="56" customHeight="1">
-      <c r="A178" s="44" t="s">
+      <c r="A178" s="6" t="s">
         <v>796</v>
       </c>
       <c r="B178" s="5" t="s">
@@ -13854,14 +13778,12 @@
       <c r="G178" s="5" t="s">
         <v>800</v>
       </c>
-      <c r="H178" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷: کانال‌های موسیقی، تماس، مسیریاب، دستیار صوتی و سیستم با AudioPolicy خودرو؛ بازه واقعی دستگاه بررسی می‌شود. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H178" s="5" t="s">
+        <v>2845</v>
       </c>
     </row>
     <row r="179" spans="1:8" ht="56" customHeight="1">
-      <c r="A179" s="45" t="s">
+      <c r="A179" s="6" t="s">
         <v>801</v>
       </c>
       <c r="B179" s="1" t="s">
@@ -13882,10 +13804,8 @@
       <c r="G179" s="1" t="s">
         <v>805</v>
       </c>
-      <c r="H179" s="1" t="inlineStr">
-        <is>
-          <t>فاز ۷: کانال‌های موسیقی، تماس، مسیریاب، دستیار صوتی و سیستم با AudioPolicy خودرو؛ بازه واقعی دستگاه بررسی می‌شود. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H179" s="1" t="s">
+        <v>2845</v>
       </c>
     </row>
     <row r="180" spans="1:8" ht="56" customHeight="1">
@@ -14227,7 +14147,7 @@
       </c>
     </row>
     <row r="193" spans="1:8" ht="56" customHeight="1">
-      <c r="A193" s="46" t="s">
+      <c r="A193" s="6" t="s">
         <v>868</v>
       </c>
       <c r="B193" s="1" t="s">
@@ -14248,14 +14168,12 @@
       <c r="G193" s="1" t="s">
         <v>871</v>
       </c>
-      <c r="H193" s="1" t="inlineStr">
-        <is>
-          <t>فاز ۷: ارسال کلید رسانه به پلیر فعال سیستم؛ رها پیش از فرمان فوکوس صدا را آزاد می‌کند. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H193" s="1" t="s">
+        <v>2846</v>
       </c>
     </row>
     <row r="194" spans="1:8" ht="56" customHeight="1">
-      <c r="A194" s="47" t="s">
+      <c r="A194" s="6" t="s">
         <v>872</v>
       </c>
       <c r="B194" s="5" t="s">
@@ -14276,14 +14194,12 @@
       <c r="G194" s="5" t="s">
         <v>871</v>
       </c>
-      <c r="H194" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷: ارسال کلید رسانه به پلیر فعال سیستم؛ رها پیش از فرمان فوکوس صدا را آزاد می‌کند. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H194" s="5" t="s">
+        <v>2846</v>
       </c>
     </row>
     <row r="195" spans="1:8" ht="56" customHeight="1">
-      <c r="A195" s="48" t="s">
+      <c r="A195" s="6" t="s">
         <v>874</v>
       </c>
       <c r="B195" s="1" t="s">
@@ -14304,14 +14220,12 @@
       <c r="G195" s="1" t="s">
         <v>877</v>
       </c>
-      <c r="H195" s="1" t="inlineStr">
-        <is>
-          <t>فاز ۷: ارسال کلید رسانه به پلیر فعال سیستم؛ رها پیش از فرمان فوکوس صدا را آزاد می‌کند. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H195" s="1" t="s">
+        <v>2846</v>
       </c>
     </row>
     <row r="196" spans="1:8" ht="56" customHeight="1">
-      <c r="A196" s="49" t="s">
+      <c r="A196" s="6" t="s">
         <v>878</v>
       </c>
       <c r="B196" s="5" t="s">
@@ -14332,10 +14246,8 @@
       <c r="G196" s="5" t="s">
         <v>881</v>
       </c>
-      <c r="H196" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷: ارسال کلید رسانه به پلیر فعال سیستم؛ رها پیش از فرمان فوکوس صدا را آزاد می‌کند. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H196" s="5" t="s">
+        <v>2846</v>
       </c>
     </row>
     <row r="197" spans="1:8" ht="56" customHeight="1">
@@ -15509,7 +15421,7 @@
       </c>
     </row>
     <row r="242" spans="1:8" ht="56" customHeight="1">
-      <c r="A242" s="50" t="s">
+      <c r="A242" s="6" t="s">
         <v>1078</v>
       </c>
       <c r="B242" s="5" t="s">
@@ -15530,14 +15442,12 @@
       <c r="G242" s="5" t="s">
         <v>1083</v>
       </c>
-      <c r="H242" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷: دوربین پیش‌فرض از مسیر اصلی اپ Camera؛ انتخاب نمای خاص اضافه نشده؛ شروط اشغال دوربین و دنده‌عقب حفظ می‌شوند. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H242" s="5" t="s">
+        <v>2847</v>
       </c>
     </row>
     <row r="243" spans="1:8" ht="56" customHeight="1">
-      <c r="A243" s="51" t="s">
+      <c r="A243" s="6" t="s">
         <v>1084</v>
       </c>
       <c r="B243" s="1" t="s">
@@ -15558,14 +15468,12 @@
       <c r="G243" s="1" t="s">
         <v>1087</v>
       </c>
-      <c r="H243" s="1" t="inlineStr">
-        <is>
-          <t>فاز ۷: دوربین پیش‌فرض از مسیر اصلی اپ Camera؛ انتخاب نمای خاص اضافه نشده؛ شروط اشغال دوربین و دنده‌عقب حفظ می‌شوند. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H243" s="1" t="s">
+        <v>2847</v>
       </c>
     </row>
     <row r="244" spans="1:8" ht="56" customHeight="1">
-      <c r="A244" s="52" t="s">
+      <c r="A244" s="6" t="s">
         <v>1088</v>
       </c>
       <c r="B244" s="5" t="s">
@@ -15586,14 +15494,12 @@
       <c r="G244" s="5" t="s">
         <v>1091</v>
       </c>
-      <c r="H244" s="5" t="inlineStr">
-        <is>
-          <t>فاز ۷: دوربین پیش‌فرض از مسیر اصلی اپ Camera؛ انتخاب نمای خاص اضافه نشده؛ شروط اشغال دوربین و دنده‌عقب حفظ می‌شوند. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H244" s="5" t="s">
+        <v>2847</v>
       </c>
     </row>
     <row r="245" spans="1:8" ht="56" customHeight="1">
-      <c r="A245" s="53" t="s">
+      <c r="A245" s="6" t="s">
         <v>1092</v>
       </c>
       <c r="B245" s="1" t="s">
@@ -15614,10 +15520,8 @@
       <c r="G245" s="1" t="s">
         <v>1095</v>
       </c>
-      <c r="H245" s="1" t="inlineStr">
-        <is>
-          <t>فاز ۷: توقف ضبط با رویداد اصلی اپ Camera؛ بدون بازکردن دوباره برنامه و بدون تبدیل توقف به شروع. نیازمند تست خودرو.</t>
-        </is>
+      <c r="H245" s="1" t="s">
+        <v>2848</v>
       </c>
     </row>
     <row r="246" spans="1:8" ht="56" customHeight="1">

</xml_diff>